<commit_message>
Limit McNemar BH correction to displayed comparisons
</commit_message>
<xml_diff>
--- a/mcnemar/SuppFile2_Stats_generated.xlsx
+++ b/mcnemar/SuppFile2_Stats_generated.xlsx
@@ -11771,7 +11771,7 @@
         <v>8</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.0745</v>
+        <v>0.124</v>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
@@ -11785,7 +11785,7 @@
         <v>8</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.06950000000000001</v>
+        <v>0.0772</v>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
@@ -11875,7 +11875,7 @@
         <v>2</v>
       </c>
       <c r="Z3" s="3" t="n">
-        <v>8.729999999999999e-05</v>
+        <v>5.82e-05</v>
       </c>
       <c r="AA3" s="3" t="inlineStr">
         <is>
@@ -11889,7 +11889,7 @@
         <v>11</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="AF3" t="inlineStr">
         <is>
@@ -12286,7 +12286,7 @@
         <v>4</v>
       </c>
       <c r="Z7" s="3" t="n">
-        <v>0.0022</v>
+        <v>0.00146</v>
       </c>
       <c r="AA7" s="3" t="inlineStr">
         <is>
@@ -12300,7 +12300,7 @@
         <v>1</v>
       </c>
       <c r="AE7" s="3" t="n">
-        <v>1.09e-05</v>
+        <v>7.29e-06</v>
       </c>
       <c r="AF7" s="3" t="inlineStr">
         <is>
@@ -12390,7 +12390,7 @@
         <v>7</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.139</v>
+        <v>0.0927</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
@@ -12400,13 +12400,13 @@
       <c r="AC8" t="n">
         <v>0.00418</v>
       </c>
-      <c r="AD8" s="4" t="n">
+      <c r="AD8" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="AE8" s="4" t="n">
-        <v>0.0125</v>
-      </c>
-      <c r="AF8" s="4" t="inlineStr">
+      <c r="AE8" s="3" t="n">
+        <v>0.008359999999999999</v>
+      </c>
+      <c r="AF8" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -12588,7 +12588,7 @@
         <v>6</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.0653</v>
+        <v>0.058</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -12692,7 +12692,7 @@
         <v>10</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.752</v>
+        <v>0.762</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -12706,7 +12706,7 @@
         <v>10</v>
       </c>
       <c r="AE11" t="n">
-        <v>0.582</v>
+        <v>0.544</v>
       </c>
       <c r="AF11" t="inlineStr">
         <is>
@@ -12796,7 +12796,7 @@
         <v>5</v>
       </c>
       <c r="Z12" s="3" t="n">
-        <v>0.00229</v>
+        <v>0.00305</v>
       </c>
       <c r="AA12" s="3" t="inlineStr">
         <is>
@@ -12810,7 +12810,7 @@
         <v>2</v>
       </c>
       <c r="AE12" s="3" t="n">
-        <v>0.000268</v>
+        <v>0.000357</v>
       </c>
       <c r="AF12" s="3" t="inlineStr">
         <is>
@@ -12900,7 +12900,7 @@
         <v>11</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.9409999999999999</v>
+        <v>1</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -12910,15 +12910,15 @@
       <c r="AC13" t="n">
         <v>0.0225</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AD13" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="AE13" t="n">
-        <v>0.0675</v>
-      </c>
-      <c r="AF13" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="AE13" s="4" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="AF13" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AH13" t="inlineStr">
@@ -13103,7 +13103,7 @@
         <v>9</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.657</v>
+        <v>0.766</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -13117,7 +13117,7 @@
         <v>6</v>
       </c>
       <c r="AE15" s="4" t="n">
-        <v>0.0333</v>
+        <v>0.0222</v>
       </c>
       <c r="AF15" s="4" t="inlineStr">
         <is>
@@ -13202,7 +13202,7 @@
         <v>3</v>
       </c>
       <c r="Z16" s="3" t="n">
-        <v>0.000109</v>
+        <v>7.29e-05</v>
       </c>
       <c r="AA16" s="3" t="inlineStr">
         <is>
@@ -13216,7 +13216,7 @@
         <v>9</v>
       </c>
       <c r="AE16" t="n">
-        <v>0.138</v>
+        <v>0.123</v>
       </c>
       <c r="AF16" t="inlineStr">
         <is>
@@ -13301,7 +13301,7 @@
         <v>1</v>
       </c>
       <c r="Z17" s="3" t="n">
-        <v>2.23e-05</v>
+        <v>1.49e-05</v>
       </c>
       <c r="AA17" s="3" t="inlineStr">
         <is>
@@ -13311,13 +13311,13 @@
       <c r="AC17" t="n">
         <v>0.00149</v>
       </c>
-      <c r="AD17" s="4" t="n">
+      <c r="AD17" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="AE17" s="4" t="n">
-        <v>0.0134</v>
-      </c>
-      <c r="AF17" s="4" t="inlineStr">
+      <c r="AE17" s="3" t="n">
+        <v>0.00894</v>
+      </c>
+      <c r="AF17" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -13415,7 +13415,7 @@
         <v>5</v>
       </c>
       <c r="AE19" t="n">
-        <v>0.08409999999999999</v>
+        <v>0.0785</v>
       </c>
       <c r="AF19" t="inlineStr">
         <is>
@@ -13500,7 +13500,7 @@
         <v>2</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.12</v>
+        <v>0.112</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -13599,7 +13599,7 @@
         <v>6</v>
       </c>
       <c r="Z21" t="n">
-        <v>1</v>
+        <v>0.908</v>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
@@ -13811,7 +13811,7 @@
         <v>10</v>
       </c>
       <c r="AE23" t="n">
-        <v>0.721</v>
+        <v>0.722</v>
       </c>
       <c r="AF23" t="inlineStr">
         <is>
@@ -13896,7 +13896,7 @@
         <v>7</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.393</v>
+        <v>0.349</v>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
@@ -13910,7 +13910,7 @@
         <v>1</v>
       </c>
       <c r="AE24" s="3" t="n">
-        <v>3.15e-05</v>
+        <v>2.1e-05</v>
       </c>
       <c r="AF24" s="3" t="inlineStr">
         <is>
@@ -13995,7 +13995,7 @@
         <v>10</v>
       </c>
       <c r="Z25" t="n">
-        <v>0.789</v>
+        <v>0.701</v>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
@@ -14009,7 +14009,7 @@
         <v>2</v>
       </c>
       <c r="AE25" s="3" t="n">
-        <v>0.00234</v>
+        <v>0.00156</v>
       </c>
       <c r="AF25" s="3" t="inlineStr">
         <is>
@@ -14094,7 +14094,7 @@
         <v>3</v>
       </c>
       <c r="Z26" t="n">
-        <v>0.49</v>
+        <v>0.327</v>
       </c>
       <c r="AA26" t="inlineStr">
         <is>
@@ -14193,7 +14193,7 @@
         <v>4</v>
       </c>
       <c r="Z27" t="n">
-        <v>0.296</v>
+        <v>0.337</v>
       </c>
       <c r="AA27" t="inlineStr">
         <is>
@@ -14391,7 +14391,7 @@
         <v>1</v>
       </c>
       <c r="Z29" t="n">
-        <v>0.117</v>
+        <v>0.13</v>
       </c>
       <c r="AA29" t="inlineStr">
         <is>
@@ -14405,7 +14405,7 @@
         <v>3</v>
       </c>
       <c r="AE29" s="3" t="n">
-        <v>0.00585</v>
+        <v>0.0078</v>
       </c>
       <c r="AF29" s="3" t="inlineStr">
         <is>
@@ -14490,7 +14490,7 @@
         <v>5</v>
       </c>
       <c r="Z30" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.996</v>
       </c>
       <c r="AA30" t="inlineStr">
         <is>
@@ -14504,7 +14504,7 @@
         <v>4</v>
       </c>
       <c r="AE30" t="n">
-        <v>0.08690000000000001</v>
+        <v>0.0579</v>
       </c>
       <c r="AF30" t="inlineStr">
         <is>
@@ -14702,7 +14702,7 @@
         <v>8</v>
       </c>
       <c r="AE32" t="n">
-        <v>0.3</v>
+        <v>0.267</v>
       </c>
       <c r="AF32" t="inlineStr">
         <is>
@@ -14787,7 +14787,7 @@
         <v>9</v>
       </c>
       <c r="Z33" t="n">
-        <v>0.768</v>
+        <v>0.716</v>
       </c>
       <c r="AA33" t="inlineStr">
         <is>
@@ -14801,7 +14801,7 @@
         <v>9</v>
       </c>
       <c r="AE33" t="n">
-        <v>0.388</v>
+        <v>0.362</v>
       </c>
       <c r="AF33" t="inlineStr">
         <is>
@@ -14900,7 +14900,7 @@
         <v>7</v>
       </c>
       <c r="AE34" t="n">
-        <v>0.498</v>
+        <v>0.429</v>
       </c>
       <c r="AF34" t="inlineStr">
         <is>
@@ -14987,7 +14987,7 @@
         <v>6</v>
       </c>
       <c r="Z37" t="n">
-        <v>0.195</v>
+        <v>0.228</v>
       </c>
       <c r="AA37" t="inlineStr">
         <is>
@@ -15001,7 +15001,7 @@
         <v>4</v>
       </c>
       <c r="AE37" t="n">
-        <v>0.08409999999999999</v>
+        <v>0.0785</v>
       </c>
       <c r="AF37" t="inlineStr">
         <is>
@@ -15100,7 +15100,7 @@
         <v>7</v>
       </c>
       <c r="AE38" t="n">
-        <v>0.45</v>
+        <v>0.75</v>
       </c>
       <c r="AF38" t="inlineStr">
         <is>
@@ -15185,7 +15185,7 @@
         <v>9</v>
       </c>
       <c r="Z39" t="n">
-        <v>1</v>
+        <v>0.908</v>
       </c>
       <c r="AA39" t="inlineStr">
         <is>
@@ -15199,7 +15199,7 @@
         <v>5</v>
       </c>
       <c r="AE39" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.681</v>
       </c>
       <c r="AF39" t="inlineStr">
         <is>
@@ -15397,7 +15397,7 @@
         <v>9</v>
       </c>
       <c r="AE41" t="n">
-        <v>0.721</v>
+        <v>0.722</v>
       </c>
       <c r="AF41" t="inlineStr">
         <is>
@@ -15482,7 +15482,7 @@
         <v>3</v>
       </c>
       <c r="Z42" t="n">
-        <v>0.0931</v>
+        <v>0.0621</v>
       </c>
       <c r="AA42" t="inlineStr">
         <is>
@@ -15496,7 +15496,7 @@
         <v>12</v>
       </c>
       <c r="AE42" t="n">
-        <v>0.618</v>
+        <v>0.549</v>
       </c>
       <c r="AF42" t="inlineStr">
         <is>
@@ -15581,7 +15581,7 @@
         <v>11</v>
       </c>
       <c r="Z43" t="n">
-        <v>0.789</v>
+        <v>0.701</v>
       </c>
       <c r="AA43" t="inlineStr">
         <is>
@@ -15680,7 +15680,7 @@
         <v>8</v>
       </c>
       <c r="Z44" t="n">
-        <v>0.844</v>
+        <v>0.75</v>
       </c>
       <c r="AA44" t="inlineStr">
         <is>
@@ -15878,7 +15878,7 @@
         <v>5</v>
       </c>
       <c r="Z46" t="n">
-        <v>0.17</v>
+        <v>0.151</v>
       </c>
       <c r="AA46" t="inlineStr">
         <is>
@@ -15892,7 +15892,7 @@
         <v>2</v>
       </c>
       <c r="AE46" t="n">
-        <v>0.0974</v>
+        <v>0.0866</v>
       </c>
       <c r="AF46" t="inlineStr">
         <is>
@@ -15991,7 +15991,7 @@
         <v>9</v>
       </c>
       <c r="AE47" t="n">
-        <v>0.545</v>
+        <v>0.636</v>
       </c>
       <c r="AF47" t="inlineStr">
         <is>
@@ -16090,7 +16090,7 @@
         <v>8</v>
       </c>
       <c r="AE48" t="n">
-        <v>0.516</v>
+        <v>0.413</v>
       </c>
       <c r="AF48" t="inlineStr">
         <is>
@@ -16288,7 +16288,7 @@
         <v>6</v>
       </c>
       <c r="AE50" t="n">
-        <v>0.3</v>
+        <v>0.267</v>
       </c>
       <c r="AF50" t="inlineStr">
         <is>
@@ -16373,7 +16373,7 @@
         <v>2</v>
       </c>
       <c r="Z51" s="3" t="n">
-        <v>0.000768</v>
+        <v>0.000512</v>
       </c>
       <c r="AA51" s="3" t="inlineStr">
         <is>
@@ -16387,7 +16387,7 @@
         <v>1</v>
       </c>
       <c r="AE51" s="3" t="n">
-        <v>0.000297</v>
+        <v>0.000396</v>
       </c>
       <c r="AF51" s="3" t="inlineStr">
         <is>
@@ -16472,7 +16472,7 @@
         <v>1</v>
       </c>
       <c r="Z52" s="3" t="n">
-        <v>1.38e-05</v>
+        <v>9.18e-06</v>
       </c>
       <c r="AA52" s="3" t="inlineStr">
         <is>
@@ -16572,7 +16572,7 @@
         <v>5</v>
       </c>
       <c r="Z54" s="4" t="n">
-        <v>0.0235</v>
+        <v>0.0313</v>
       </c>
       <c r="AA54" s="4" t="inlineStr">
         <is>
@@ -16671,7 +16671,7 @@
         <v>3</v>
       </c>
       <c r="Z55" s="3" t="n">
-        <v>6.87e-05</v>
+        <v>4.58e-05</v>
       </c>
       <c r="AA55" s="3" t="inlineStr">
         <is>
@@ -16770,7 +16770,7 @@
         <v>11</v>
       </c>
       <c r="Z56" t="n">
-        <v>1</v>
+        <v>0.908</v>
       </c>
       <c r="AA56" t="inlineStr">
         <is>
@@ -16883,7 +16883,7 @@
         <v>9</v>
       </c>
       <c r="AE57" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="AF57" t="inlineStr">
         <is>
@@ -16982,7 +16982,7 @@
         <v>8</v>
       </c>
       <c r="AE58" t="n">
-        <v>0.721</v>
+        <v>0.722</v>
       </c>
       <c r="AF58" t="inlineStr">
         <is>
@@ -17067,7 +17067,7 @@
         <v>4</v>
       </c>
       <c r="Z59" s="3" t="n">
-        <v>0.0022</v>
+        <v>0.00146</v>
       </c>
       <c r="AA59" s="3" t="inlineStr">
         <is>
@@ -17081,7 +17081,7 @@
         <v>6</v>
       </c>
       <c r="AE59" s="4" t="n">
-        <v>0.0405</v>
+        <v>0.0338</v>
       </c>
       <c r="AF59" s="4" t="inlineStr">
         <is>
@@ -17162,15 +17162,15 @@
       <c r="X60" t="n">
         <v>0.0072</v>
       </c>
-      <c r="Y60" t="n">
+      <c r="Y60" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="Z60" t="n">
-        <v>0.0648</v>
-      </c>
-      <c r="AA60" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="Z60" s="4" t="n">
+        <v>0.0432</v>
+      </c>
+      <c r="AA60" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AC60" t="n">
@@ -17180,7 +17180,7 @@
         <v>5</v>
       </c>
       <c r="AE60" s="4" t="n">
-        <v>0.0263</v>
+        <v>0.0175</v>
       </c>
       <c r="AF60" s="4" t="inlineStr">
         <is>
@@ -17378,7 +17378,7 @@
         <v>4</v>
       </c>
       <c r="AE62" s="4" t="n">
-        <v>0.0149</v>
+        <v>0.0132</v>
       </c>
       <c r="AF62" s="4" t="inlineStr">
         <is>
@@ -17477,7 +17477,7 @@
         <v>2</v>
       </c>
       <c r="AE63" s="4" t="n">
-        <v>0.0367</v>
+        <v>0.0245</v>
       </c>
       <c r="AF63" s="4" t="inlineStr">
         <is>
@@ -17576,7 +17576,7 @@
         <v>11</v>
       </c>
       <c r="AE64" t="n">
-        <v>0.763</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="AF64" t="inlineStr">
         <is>
@@ -17661,7 +17661,7 @@
         <v>10</v>
       </c>
       <c r="Z65" t="n">
-        <v>0.472</v>
+        <v>0.315</v>
       </c>
       <c r="AA65" t="inlineStr">
         <is>
@@ -17675,7 +17675,7 @@
         <v>3</v>
       </c>
       <c r="AE65" s="4" t="n">
-        <v>0.0286</v>
+        <v>0.019</v>
       </c>
       <c r="AF65" s="4" t="inlineStr">
         <is>
@@ -17873,7 +17873,7 @@
         <v>7</v>
       </c>
       <c r="AE67" t="n">
-        <v>0.3</v>
+        <v>0.267</v>
       </c>
       <c r="AF67" t="inlineStr">
         <is>
@@ -17958,7 +17958,7 @@
         <v>2</v>
       </c>
       <c r="Z68" s="3" t="n">
-        <v>9.989999999999999e-06</v>
+        <v>6.66e-06</v>
       </c>
       <c r="AA68" s="3" t="inlineStr">
         <is>
@@ -17972,7 +17972,7 @@
         <v>11</v>
       </c>
       <c r="AE68" t="n">
-        <v>0.763</v>
+        <v>0.678</v>
       </c>
       <c r="AF68" t="inlineStr">
         <is>
@@ -18057,7 +18057,7 @@
         <v>1</v>
       </c>
       <c r="Z69" s="3" t="n">
-        <v>8.019999999999999e-06</v>
+        <v>5.35e-06</v>
       </c>
       <c r="AA69" s="3" t="inlineStr">
         <is>
@@ -18158,7 +18158,7 @@
         <v>5</v>
       </c>
       <c r="Z72" t="n">
-        <v>0.195</v>
+        <v>0.228</v>
       </c>
       <c r="AA72" t="inlineStr">
         <is>
@@ -18271,7 +18271,7 @@
         <v>3</v>
       </c>
       <c r="AE73" t="n">
-        <v>0.211</v>
+        <v>0.375</v>
       </c>
       <c r="AF73" t="inlineStr">
         <is>
@@ -18455,7 +18455,7 @@
         <v>6</v>
       </c>
       <c r="Z75" t="n">
-        <v>0.54</v>
+        <v>1</v>
       </c>
       <c r="AA75" t="inlineStr">
         <is>
@@ -18469,7 +18469,7 @@
         <v>8</v>
       </c>
       <c r="AE75" t="n">
-        <v>0.54</v>
+        <v>1</v>
       </c>
       <c r="AF75" t="inlineStr">
         <is>
@@ -18653,7 +18653,7 @@
         <v>7</v>
       </c>
       <c r="Z77" t="n">
-        <v>0.381</v>
+        <v>0.322</v>
       </c>
       <c r="AA77" t="inlineStr">
         <is>
@@ -18667,7 +18667,7 @@
         <v>4</v>
       </c>
       <c r="AE77" t="n">
-        <v>0.0978</v>
+        <v>0.07820000000000001</v>
       </c>
       <c r="AF77" t="inlineStr">
         <is>
@@ -18752,7 +18752,7 @@
         <v>9</v>
       </c>
       <c r="Z78" t="n">
-        <v>0.789</v>
+        <v>0.701</v>
       </c>
       <c r="AA78" t="inlineStr">
         <is>
@@ -18766,7 +18766,7 @@
         <v>7</v>
       </c>
       <c r="AE78" t="n">
-        <v>0.217</v>
+        <v>0.203</v>
       </c>
       <c r="AF78" t="inlineStr">
         <is>
@@ -18964,7 +18964,7 @@
         <v>11</v>
       </c>
       <c r="AE80" t="n">
-        <v>0.273</v>
+        <v>0.292</v>
       </c>
       <c r="AF80" t="inlineStr">
         <is>
@@ -19063,7 +19063,7 @@
         <v>2</v>
       </c>
       <c r="AE81" t="n">
-        <v>0.0974</v>
+        <v>0.0866</v>
       </c>
       <c r="AF81" t="inlineStr">
         <is>
@@ -19162,7 +19162,7 @@
         <v>5</v>
       </c>
       <c r="AE82" t="n">
-        <v>0.201</v>
+        <v>0.268</v>
       </c>
       <c r="AF82" t="inlineStr">
         <is>
@@ -19360,7 +19360,7 @@
         <v>1</v>
       </c>
       <c r="AE84" t="n">
-        <v>0.176</v>
+        <v>0.187</v>
       </c>
       <c r="AF84" t="inlineStr">
         <is>
@@ -19445,7 +19445,7 @@
         <v>11</v>
       </c>
       <c r="Z85" t="n">
-        <v>0.657</v>
+        <v>0.766</v>
       </c>
       <c r="AA85" t="inlineStr">
         <is>
@@ -19459,7 +19459,7 @@
         <v>12</v>
       </c>
       <c r="AE85" t="n">
-        <v>0.3</v>
+        <v>0.267</v>
       </c>
       <c r="AF85" t="inlineStr">
         <is>
@@ -19544,7 +19544,7 @@
         <v>4</v>
       </c>
       <c r="Z86" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.0733</v>
       </c>
       <c r="AA86" t="inlineStr">
         <is>
@@ -19643,7 +19643,7 @@
         <v>1</v>
       </c>
       <c r="Z87" s="4" t="n">
-        <v>0.014</v>
+        <v>0.0117</v>
       </c>
       <c r="AA87" s="4" t="inlineStr">
         <is>
@@ -19657,7 +19657,7 @@
         <v>13</v>
       </c>
       <c r="AE87" t="n">
-        <v>0.498</v>
+        <v>0.429</v>
       </c>
       <c r="AF87" t="inlineStr">
         <is>
@@ -19743,7 +19743,7 @@
         <v>7</v>
       </c>
       <c r="Z89" t="n">
-        <v>0.461</v>
+        <v>0.492</v>
       </c>
       <c r="AA89" t="inlineStr">
         <is>
@@ -19757,7 +19757,7 @@
         <v>3</v>
       </c>
       <c r="AE89" s="3" t="n">
-        <v>4.29e-06</v>
+        <v>5.72e-06</v>
       </c>
       <c r="AF89" s="3" t="inlineStr">
         <is>
@@ -19842,7 +19842,7 @@
         <v>2</v>
       </c>
       <c r="Z90" s="3" t="n">
-        <v>0.0012</v>
+        <v>0.00107</v>
       </c>
       <c r="AA90" s="3" t="inlineStr">
         <is>
@@ -19955,7 +19955,7 @@
         <v>10</v>
       </c>
       <c r="AE91" t="n">
-        <v>0.844</v>
+        <v>0.75</v>
       </c>
       <c r="AF91" t="inlineStr">
         <is>
@@ -20054,7 +20054,7 @@
         <v>11</v>
       </c>
       <c r="AE92" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="AF92" t="inlineStr">
         <is>
@@ -20153,7 +20153,7 @@
         <v>7</v>
       </c>
       <c r="AE93" s="4" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AF93" s="4" t="inlineStr">
         <is>
@@ -20238,7 +20238,7 @@
         <v>4</v>
       </c>
       <c r="Z94" t="n">
-        <v>0.0931</v>
+        <v>0.0621</v>
       </c>
       <c r="AA94" t="inlineStr">
         <is>
@@ -20252,7 +20252,7 @@
         <v>4</v>
       </c>
       <c r="AE94" s="3" t="n">
-        <v>1.09e-05</v>
+        <v>7.29e-06</v>
       </c>
       <c r="AF94" s="3" t="inlineStr">
         <is>
@@ -20337,7 +20337,7 @@
         <v>8</v>
       </c>
       <c r="Z95" t="n">
-        <v>0.789</v>
+        <v>0.701</v>
       </c>
       <c r="AA95" t="inlineStr">
         <is>
@@ -20351,7 +20351,7 @@
         <v>2</v>
       </c>
       <c r="AE95" s="3" t="n">
-        <v>4.29e-06</v>
+        <v>2.86e-06</v>
       </c>
       <c r="AF95" s="3" t="inlineStr">
         <is>
@@ -20432,13 +20432,13 @@
       <c r="X96" t="n">
         <v>0.00149</v>
       </c>
-      <c r="Y96" s="4" t="n">
+      <c r="Y96" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="Z96" s="4" t="n">
-        <v>0.0134</v>
-      </c>
-      <c r="AA96" s="4" t="inlineStr">
+      <c r="Z96" s="3" t="n">
+        <v>0.00894</v>
+      </c>
+      <c r="AA96" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -20535,7 +20535,7 @@
         <v>1</v>
       </c>
       <c r="Z97" s="3" t="n">
-        <v>0.000555</v>
+        <v>0.00037</v>
       </c>
       <c r="AA97" s="3" t="inlineStr">
         <is>
@@ -20549,7 +20549,7 @@
         <v>1</v>
       </c>
       <c r="AE97" s="3" t="n">
-        <v>3.99e-06</v>
+        <v>2.66e-06</v>
       </c>
       <c r="AF97" s="3" t="inlineStr">
         <is>
@@ -20648,7 +20648,7 @@
         <v>9</v>
       </c>
       <c r="AE98" t="n">
-        <v>0.46</v>
+        <v>0.461</v>
       </c>
       <c r="AF98" t="inlineStr">
         <is>
@@ -20733,7 +20733,7 @@
         <v>5</v>
       </c>
       <c r="Z99" t="n">
-        <v>0.117</v>
+        <v>0.13</v>
       </c>
       <c r="AA99" t="inlineStr">
         <is>
@@ -20846,7 +20846,7 @@
         <v>5</v>
       </c>
       <c r="AE100" s="3" t="n">
-        <v>9.899999999999999e-05</v>
+        <v>6.600000000000001e-05</v>
       </c>
       <c r="AF100" s="3" t="inlineStr">
         <is>
@@ -21030,7 +21030,7 @@
         <v>10</v>
       </c>
       <c r="Z102" t="n">
-        <v>0.763</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="AA102" t="inlineStr">
         <is>
@@ -21044,7 +21044,7 @@
         <v>6</v>
       </c>
       <c r="AE102" s="3" t="n">
-        <v>0.000687</v>
+        <v>0.000458</v>
       </c>
       <c r="AF102" s="3" t="inlineStr">
         <is>
@@ -21143,7 +21143,7 @@
         <v>8</v>
       </c>
       <c r="AE103" t="n">
-        <v>0.138</v>
+        <v>0.123</v>
       </c>
       <c r="AF103" t="inlineStr">
         <is>
@@ -21228,7 +21228,7 @@
         <v>9</v>
       </c>
       <c r="Z104" t="n">
-        <v>0.73</v>
+        <v>0.779</v>
       </c>
       <c r="AA104" t="inlineStr">
         <is>
@@ -21242,7 +21242,7 @@
         <v>14</v>
       </c>
       <c r="AE104" t="n">
-        <v>0.836</v>
+        <v>0.86</v>
       </c>
       <c r="AF104" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Limit Fisher BH correction to displayed comparisons
</commit_message>
<xml_diff>
--- a/mcnemar/SuppFile2_Stats_generated.xlsx
+++ b/mcnemar/SuppFile2_Stats_generated.xlsx
@@ -708,7 +708,7 @@
         <v>7</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.18</v>
+        <v>0.3</v>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
@@ -722,7 +722,7 @@
         <v>9</v>
       </c>
       <c r="AE2" t="n">
-        <v>1</v>
+        <v>0.965</v>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
@@ -736,7 +736,7 @@
         <v>8</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.175</v>
+        <v>0.195</v>
       </c>
       <c r="AK2" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
         <v>1</v>
       </c>
       <c r="Z3" s="3" t="n">
-        <v>0.000782</v>
+        <v>0.000521</v>
       </c>
       <c r="AA3" s="3" t="inlineStr">
         <is>
@@ -840,7 +840,7 @@
         <v>1</v>
       </c>
       <c r="AE3" s="3" t="n">
-        <v>0.00524</v>
+        <v>0.00349</v>
       </c>
       <c r="AF3" s="3" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
         <v>10</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.736</v>
+        <v>0.982</v>
       </c>
       <c r="AK3" t="inlineStr">
         <is>
@@ -1293,7 +1293,7 @@
         <v>5</v>
       </c>
       <c r="Z7" s="4" t="n">
-        <v>0.0352</v>
+        <v>0.0235</v>
       </c>
       <c r="AA7" s="4" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
         <v>1</v>
       </c>
       <c r="AJ7" s="3" t="n">
-        <v>0.000488</v>
+        <v>0.000434</v>
       </c>
       <c r="AK7" s="3" t="inlineStr">
         <is>
@@ -1411,7 +1411,7 @@
         <v>6</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.41</v>
+        <v>0.273</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
@@ -1425,7 +1425,7 @@
         <v>11</v>
       </c>
       <c r="AE8" t="n">
-        <v>0.754</v>
+        <v>0.729</v>
       </c>
       <c r="AF8" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         <v>4</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.0423</v>
+        <v>0.0282</v>
       </c>
       <c r="AK8" s="4" t="inlineStr">
         <is>
@@ -1637,7 +1637,7 @@
         <v>8</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.367</v>
+        <v>0.326</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         <v>5</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.858</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="AF10" t="inlineStr">
         <is>
@@ -1783,7 +1783,7 @@
         <v>11</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.776</v>
+        <v>0.828</v>
       </c>
       <c r="AK11" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
         <v>4</v>
       </c>
       <c r="Z12" s="4" t="n">
-        <v>0.0239</v>
+        <v>0.0319</v>
       </c>
       <c r="AA12" s="4" t="inlineStr">
         <is>
@@ -1887,7 +1887,7 @@
         <v>8</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.721</v>
+        <v>0.769</v>
       </c>
       <c r="AF12" t="inlineStr">
         <is>
@@ -1897,13 +1897,13 @@
       <c r="AH12" t="n">
         <v>0.00195</v>
       </c>
-      <c r="AI12" s="3" t="n">
+      <c r="AI12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="AJ12" s="3" t="n">
-        <v>0.00877</v>
-      </c>
-      <c r="AK12" s="3" t="inlineStr">
+      <c r="AJ12" s="4" t="n">
+        <v>0.0117</v>
+      </c>
+      <c r="AK12" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -2005,7 +2005,7 @@
         <v>6</v>
       </c>
       <c r="AE13" t="n">
-        <v>0.529</v>
+        <v>0.582</v>
       </c>
       <c r="AF13" t="inlineStr">
         <is>
@@ -2019,7 +2019,7 @@
         <v>7</v>
       </c>
       <c r="AJ13" t="n">
-        <v>0.188</v>
+        <v>0.125</v>
       </c>
       <c r="AK13" t="inlineStr">
         <is>
@@ -2222,7 +2222,7 @@
         <v>9</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.744</v>
+        <v>0.829</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -2236,7 +2236,7 @@
         <v>4</v>
       </c>
       <c r="AE15" t="n">
-        <v>0.238</v>
+        <v>0.222</v>
       </c>
       <c r="AF15" t="inlineStr">
         <is>
@@ -2250,7 +2250,7 @@
         <v>5</v>
       </c>
       <c r="AJ15" t="n">
-        <v>0.09719999999999999</v>
+        <v>0.0648</v>
       </c>
       <c r="AK15" t="inlineStr">
         <is>
@@ -2335,7 +2335,7 @@
         <v>2</v>
       </c>
       <c r="Z16" s="3" t="n">
-        <v>0.00152</v>
+        <v>0.00101</v>
       </c>
       <c r="AA16" s="3" t="inlineStr">
         <is>
@@ -2349,7 +2349,7 @@
         <v>2</v>
       </c>
       <c r="AE16" s="3" t="n">
-        <v>0.00763</v>
+        <v>0.00678</v>
       </c>
       <c r="AF16" s="3" t="inlineStr">
         <is>
@@ -2363,7 +2363,7 @@
         <v>9</v>
       </c>
       <c r="AJ16" t="n">
-        <v>0.279</v>
+        <v>0.31</v>
       </c>
       <c r="AK16" t="inlineStr">
         <is>
@@ -2448,7 +2448,7 @@
         <v>3</v>
       </c>
       <c r="Z17" s="3" t="n">
-        <v>0.00182</v>
+        <v>0.00162</v>
       </c>
       <c r="AA17" s="3" t="inlineStr">
         <is>
@@ -2462,7 +2462,7 @@
         <v>3</v>
       </c>
       <c r="AE17" s="4" t="n">
-        <v>0.0143</v>
+        <v>0.0127</v>
       </c>
       <c r="AF17" s="4" t="inlineStr">
         <is>
@@ -2575,7 +2575,7 @@
         <v>10</v>
       </c>
       <c r="AE19" t="n">
-        <v>1</v>
+        <v>0.965</v>
       </c>
       <c r="AF19" t="inlineStr">
         <is>
@@ -2589,7 +2589,7 @@
         <v>5</v>
       </c>
       <c r="AJ19" t="n">
-        <v>0.213</v>
+        <v>0.249</v>
       </c>
       <c r="AK19" t="inlineStr">
         <is>
@@ -2688,7 +2688,7 @@
         <v>7</v>
       </c>
       <c r="AE20" t="n">
-        <v>0.588</v>
+        <v>0.523</v>
       </c>
       <c r="AF20" t="inlineStr">
         <is>
@@ -2787,7 +2787,7 @@
         <v>4</v>
       </c>
       <c r="Z21" t="n">
-        <v>1</v>
+        <v>0.976</v>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
@@ -3027,7 +3027,7 @@
         <v>11</v>
       </c>
       <c r="AE23" t="n">
-        <v>1</v>
+        <v>0.998</v>
       </c>
       <c r="AF23" t="inlineStr">
         <is>
@@ -3126,7 +3126,7 @@
         <v>5</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.414</v>
+        <v>0.368</v>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
@@ -3154,7 +3154,7 @@
         <v>1</v>
       </c>
       <c r="AJ24" s="3" t="n">
-        <v>0.000104</v>
+        <v>6.96e-05</v>
       </c>
       <c r="AK24" s="3" t="inlineStr">
         <is>
@@ -3239,7 +3239,7 @@
         <v>10</v>
       </c>
       <c r="Z25" t="n">
-        <v>0.84</v>
+        <v>0.747</v>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
@@ -3263,13 +3263,13 @@
       <c r="AH25" t="n">
         <v>0.00231</v>
       </c>
-      <c r="AI25" s="4" t="n">
+      <c r="AI25" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="AJ25" s="4" t="n">
-        <v>0.0104</v>
-      </c>
-      <c r="AK25" s="4" t="inlineStr">
+      <c r="AJ25" s="3" t="n">
+        <v>0.00693</v>
+      </c>
+      <c r="AK25" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -3352,7 +3352,7 @@
         <v>2</v>
       </c>
       <c r="Z26" t="n">
-        <v>0.891</v>
+        <v>0.594</v>
       </c>
       <c r="AA26" t="inlineStr">
         <is>
@@ -3366,7 +3366,7 @@
         <v>3</v>
       </c>
       <c r="AE26" t="n">
-        <v>1</v>
+        <v>0.828</v>
       </c>
       <c r="AF26" t="inlineStr">
         <is>
@@ -3479,7 +3479,7 @@
         <v>12</v>
       </c>
       <c r="AE27" t="n">
-        <v>0.858</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="AF27" t="inlineStr">
         <is>
@@ -3493,7 +3493,7 @@
         <v>7</v>
       </c>
       <c r="AJ27" t="n">
-        <v>0.423</v>
+        <v>0.436</v>
       </c>
       <c r="AK27" t="inlineStr">
         <is>
@@ -3691,7 +3691,7 @@
         <v>1</v>
       </c>
       <c r="Z29" t="n">
-        <v>0.335</v>
+        <v>0.372</v>
       </c>
       <c r="AA29" t="inlineStr">
         <is>
@@ -3719,7 +3719,7 @@
         <v>3</v>
       </c>
       <c r="AJ29" t="n">
-        <v>0.0911</v>
+        <v>0.121</v>
       </c>
       <c r="AK29" t="inlineStr">
         <is>
@@ -3818,7 +3818,7 @@
         <v>6</v>
       </c>
       <c r="AE30" t="n">
-        <v>0.548</v>
+        <v>0.582</v>
       </c>
       <c r="AF30" t="inlineStr">
         <is>
@@ -3832,7 +3832,7 @@
         <v>4</v>
       </c>
       <c r="AJ30" t="n">
-        <v>0.247</v>
+        <v>0.165</v>
       </c>
       <c r="AK30" t="inlineStr">
         <is>
@@ -4044,7 +4044,7 @@
         <v>5</v>
       </c>
       <c r="AE32" t="n">
-        <v>0.319</v>
+        <v>0.284</v>
       </c>
       <c r="AF32" t="inlineStr">
         <is>
@@ -4058,7 +4058,7 @@
         <v>9</v>
       </c>
       <c r="AJ32" t="n">
-        <v>0.503</v>
+        <v>0.447</v>
       </c>
       <c r="AK32" t="inlineStr">
         <is>
@@ -4143,7 +4143,7 @@
         <v>9</v>
       </c>
       <c r="Z33" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.847</v>
       </c>
       <c r="AA33" t="inlineStr">
         <is>
@@ -4157,7 +4157,7 @@
         <v>7</v>
       </c>
       <c r="AE33" t="n">
-        <v>0.523</v>
+        <v>0.55</v>
       </c>
       <c r="AF33" t="inlineStr">
         <is>
@@ -4171,7 +4171,7 @@
         <v>8</v>
       </c>
       <c r="AJ33" t="n">
-        <v>0.408</v>
+        <v>0.363</v>
       </c>
       <c r="AK33" t="inlineStr">
         <is>
@@ -4284,7 +4284,7 @@
         <v>6</v>
       </c>
       <c r="AJ34" t="n">
-        <v>0.224</v>
+        <v>0.209</v>
       </c>
       <c r="AK34" t="inlineStr">
         <is>
@@ -4369,7 +4369,7 @@
         <v>6</v>
       </c>
       <c r="Z37" t="n">
-        <v>0.409</v>
+        <v>0.468</v>
       </c>
       <c r="AA37" t="inlineStr">
         <is>
@@ -4397,7 +4397,7 @@
         <v>6</v>
       </c>
       <c r="AJ37" t="n">
-        <v>0.271</v>
+        <v>0.289</v>
       </c>
       <c r="AK37" t="inlineStr">
         <is>
@@ -4496,7 +4496,7 @@
         <v>11</v>
       </c>
       <c r="AE38" t="n">
-        <v>0.588</v>
+        <v>0.523</v>
       </c>
       <c r="AF38" t="inlineStr">
         <is>
@@ -4510,7 +4510,7 @@
         <v>5</v>
       </c>
       <c r="AJ38" t="n">
-        <v>0.425</v>
+        <v>0.708</v>
       </c>
       <c r="AK38" t="inlineStr">
         <is>
@@ -4595,7 +4595,7 @@
         <v>7</v>
       </c>
       <c r="Z39" t="n">
-        <v>1</v>
+        <v>0.976</v>
       </c>
       <c r="AA39" t="inlineStr">
         <is>
@@ -4609,7 +4609,7 @@
         <v>5</v>
       </c>
       <c r="AE39" t="n">
-        <v>0.28</v>
+        <v>0.374</v>
       </c>
       <c r="AF39" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
         <v>4</v>
       </c>
       <c r="AJ39" t="n">
-        <v>0.455</v>
+        <v>0.606</v>
       </c>
       <c r="AK39" t="inlineStr">
         <is>
@@ -4934,7 +4934,7 @@
         <v>4</v>
       </c>
       <c r="Z42" t="n">
-        <v>0.293</v>
+        <v>0.244</v>
       </c>
       <c r="AA42" t="inlineStr">
         <is>
@@ -4962,7 +4962,7 @@
         <v>13</v>
       </c>
       <c r="AJ42" t="n">
-        <v>0.727</v>
+        <v>0.713</v>
       </c>
       <c r="AK42" t="inlineStr">
         <is>
@@ -5047,7 +5047,7 @@
         <v>11</v>
       </c>
       <c r="Z43" t="n">
-        <v>0.84</v>
+        <v>0.747</v>
       </c>
       <c r="AA43" t="inlineStr">
         <is>
@@ -5287,7 +5287,7 @@
         <v>10</v>
       </c>
       <c r="AE45" t="n">
-        <v>0.858</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="AF45" t="inlineStr">
         <is>
@@ -5386,7 +5386,7 @@
         <v>5</v>
       </c>
       <c r="Z46" t="n">
-        <v>0.396</v>
+        <v>0.352</v>
       </c>
       <c r="AA46" t="inlineStr">
         <is>
@@ -5414,7 +5414,7 @@
         <v>3</v>
       </c>
       <c r="AJ46" t="n">
-        <v>0.229</v>
+        <v>0.204</v>
       </c>
       <c r="AK46" t="inlineStr">
         <is>
@@ -5513,7 +5513,7 @@
         <v>4</v>
       </c>
       <c r="AE47" t="n">
-        <v>0.17</v>
+        <v>0.113</v>
       </c>
       <c r="AF47" t="inlineStr">
         <is>
@@ -5527,7 +5527,7 @@
         <v>8</v>
       </c>
       <c r="AJ47" t="n">
-        <v>0.656</v>
+        <v>0.752</v>
       </c>
       <c r="AK47" t="inlineStr">
         <is>
@@ -5626,7 +5626,7 @@
         <v>7</v>
       </c>
       <c r="AE48" t="n">
-        <v>0.279</v>
+        <v>0.372</v>
       </c>
       <c r="AF48" t="inlineStr">
         <is>
@@ -5640,7 +5640,7 @@
         <v>10</v>
       </c>
       <c r="AJ48" t="n">
-        <v>0.852</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="AK48" t="inlineStr">
         <is>
@@ -5852,7 +5852,7 @@
         <v>1</v>
       </c>
       <c r="AE50" s="3" t="n">
-        <v>0.0024</v>
+        <v>0.0032</v>
       </c>
       <c r="AF50" s="3" t="inlineStr">
         <is>
@@ -5866,7 +5866,7 @@
         <v>7</v>
       </c>
       <c r="AJ50" t="n">
-        <v>0.503</v>
+        <v>0.447</v>
       </c>
       <c r="AK50" t="inlineStr">
         <is>
@@ -5951,7 +5951,7 @@
         <v>2</v>
       </c>
       <c r="Z51" s="3" t="n">
-        <v>0.000954</v>
+        <v>0.000636</v>
       </c>
       <c r="AA51" s="3" t="inlineStr">
         <is>
@@ -5965,7 +5965,7 @@
         <v>2</v>
       </c>
       <c r="AE51" s="3" t="n">
-        <v>0.0016</v>
+        <v>0.00161</v>
       </c>
       <c r="AF51" s="3" t="inlineStr">
         <is>
@@ -5979,7 +5979,7 @@
         <v>1</v>
       </c>
       <c r="AJ51" s="3" t="n">
-        <v>0.00124</v>
+        <v>0.00165</v>
       </c>
       <c r="AK51" s="3" t="inlineStr">
         <is>
@@ -6064,7 +6064,7 @@
         <v>1</v>
       </c>
       <c r="Z52" s="3" t="n">
-        <v>1.2e-05</v>
+        <v>8.01e-06</v>
       </c>
       <c r="AA52" s="3" t="inlineStr">
         <is>
@@ -6092,7 +6092,7 @@
         <v>2</v>
       </c>
       <c r="AJ52" s="4" t="n">
-        <v>0.0372</v>
+        <v>0.0414</v>
       </c>
       <c r="AK52" s="4" t="inlineStr">
         <is>
@@ -6177,7 +6177,7 @@
         <v>5</v>
       </c>
       <c r="Z54" t="n">
-        <v>0.08790000000000001</v>
+        <v>0.129</v>
       </c>
       <c r="AA54" t="inlineStr">
         <is>
@@ -6191,7 +6191,7 @@
         <v>11</v>
       </c>
       <c r="AE54" t="n">
-        <v>1</v>
+        <v>0.965</v>
       </c>
       <c r="AF54" t="inlineStr">
         <is>
@@ -6290,7 +6290,7 @@
         <v>3</v>
       </c>
       <c r="Z55" s="3" t="n">
-        <v>0.00364</v>
+        <v>0.00486</v>
       </c>
       <c r="AA55" s="3" t="inlineStr">
         <is>
@@ -6403,7 +6403,7 @@
         <v>11</v>
       </c>
       <c r="Z56" t="n">
-        <v>1</v>
+        <v>0.976</v>
       </c>
       <c r="AA56" t="inlineStr">
         <is>
@@ -6417,7 +6417,7 @@
         <v>7</v>
       </c>
       <c r="AE56" t="n">
-        <v>0.727</v>
+        <v>0.738</v>
       </c>
       <c r="AF56" t="inlineStr">
         <is>
@@ -6544,7 +6544,7 @@
         <v>10</v>
       </c>
       <c r="AJ57" t="n">
-        <v>0.878</v>
+        <v>0.976</v>
       </c>
       <c r="AK57" t="inlineStr">
         <is>
@@ -6742,7 +6742,7 @@
         <v>4</v>
       </c>
       <c r="Z59" s="4" t="n">
-        <v>0.0352</v>
+        <v>0.0235</v>
       </c>
       <c r="AA59" s="4" t="inlineStr">
         <is>
@@ -6756,7 +6756,7 @@
         <v>4</v>
       </c>
       <c r="AE59" s="4" t="n">
-        <v>0.0394</v>
+        <v>0.035</v>
       </c>
       <c r="AF59" s="4" t="inlineStr">
         <is>
@@ -6770,7 +6770,7 @@
         <v>8</v>
       </c>
       <c r="AJ59" t="n">
-        <v>0.17</v>
+        <v>0.136</v>
       </c>
       <c r="AK59" t="inlineStr">
         <is>
@@ -6855,7 +6855,7 @@
         <v>6</v>
       </c>
       <c r="Z60" t="n">
-        <v>0.268</v>
+        <v>0.179</v>
       </c>
       <c r="AA60" t="inlineStr">
         <is>
@@ -6883,7 +6883,7 @@
         <v>4</v>
       </c>
       <c r="AJ60" t="n">
-        <v>0.108</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="AK60" t="inlineStr">
         <is>
@@ -7081,7 +7081,7 @@
         <v>10</v>
       </c>
       <c r="Z62" t="n">
-        <v>0.367</v>
+        <v>0.326</v>
       </c>
       <c r="AA62" t="inlineStr">
         <is>
@@ -7109,7 +7109,7 @@
         <v>6</v>
       </c>
       <c r="AJ62" t="n">
-        <v>0.175</v>
+        <v>0.155</v>
       </c>
       <c r="AK62" t="inlineStr">
         <is>
@@ -7222,7 +7222,7 @@
         <v>2</v>
       </c>
       <c r="AJ63" t="n">
-        <v>0.0702</v>
+        <v>0.08939999999999999</v>
       </c>
       <c r="AK63" t="inlineStr">
         <is>
@@ -7321,7 +7321,7 @@
         <v>9</v>
       </c>
       <c r="AE64" t="n">
-        <v>0.721</v>
+        <v>0.769</v>
       </c>
       <c r="AF64" t="inlineStr">
         <is>
@@ -7420,7 +7420,7 @@
         <v>9</v>
       </c>
       <c r="Z65" t="n">
-        <v>1</v>
+        <v>0.756</v>
       </c>
       <c r="AA65" t="inlineStr">
         <is>
@@ -7448,7 +7448,7 @@
         <v>3</v>
       </c>
       <c r="AJ65" t="n">
-        <v>0.188</v>
+        <v>0.125</v>
       </c>
       <c r="AK65" t="inlineStr">
         <is>
@@ -7646,7 +7646,7 @@
         <v>7</v>
       </c>
       <c r="Z67" t="n">
-        <v>0.309</v>
+        <v>0.28</v>
       </c>
       <c r="AA67" t="inlineStr">
         <is>
@@ -7660,7 +7660,7 @@
         <v>5</v>
       </c>
       <c r="AE67" t="n">
-        <v>0.181</v>
+        <v>0.204</v>
       </c>
       <c r="AF67" t="inlineStr">
         <is>
@@ -7674,7 +7674,7 @@
         <v>9</v>
       </c>
       <c r="AJ67" t="n">
-        <v>0.503</v>
+        <v>0.447</v>
       </c>
       <c r="AK67" t="inlineStr">
         <is>
@@ -7759,7 +7759,7 @@
         <v>2</v>
       </c>
       <c r="Z68" s="3" t="n">
-        <v>1.83e-05</v>
+        <v>1.22e-05</v>
       </c>
       <c r="AA68" s="3" t="inlineStr">
         <is>
@@ -7773,7 +7773,7 @@
         <v>1</v>
       </c>
       <c r="AE68" s="3" t="n">
-        <v>0.000927</v>
+        <v>0.000618</v>
       </c>
       <c r="AF68" s="3" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
         <v>5</v>
       </c>
       <c r="AJ68" t="n">
-        <v>0.137</v>
+        <v>0.183</v>
       </c>
       <c r="AK68" t="inlineStr">
         <is>
@@ -7872,7 +7872,7 @@
         <v>1</v>
       </c>
       <c r="Z69" s="3" t="n">
-        <v>6.9e-06</v>
+        <v>4.6e-06</v>
       </c>
       <c r="AA69" s="3" t="inlineStr">
         <is>
@@ -7886,7 +7886,7 @@
         <v>2</v>
       </c>
       <c r="AE69" s="3" t="n">
-        <v>0.00348</v>
+        <v>0.00351</v>
       </c>
       <c r="AF69" s="3" t="inlineStr">
         <is>
@@ -7900,7 +7900,7 @@
         <v>7</v>
       </c>
       <c r="AJ69" t="n">
-        <v>0.177</v>
+        <v>0.175</v>
       </c>
       <c r="AK69" t="inlineStr">
         <is>
@@ -7985,7 +7985,7 @@
         <v>6</v>
       </c>
       <c r="Z72" t="n">
-        <v>0.409</v>
+        <v>0.468</v>
       </c>
       <c r="AA72" t="inlineStr">
         <is>
@@ -7999,7 +7999,7 @@
         <v>11</v>
       </c>
       <c r="AE72" t="n">
-        <v>1</v>
+        <v>0.965</v>
       </c>
       <c r="AF72" t="inlineStr">
         <is>
@@ -8108,15 +8108,15 @@
       <c r="AC73" t="n">
         <v>0.0264</v>
       </c>
-      <c r="AD73" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE73" s="4" t="n">
-        <v>0.0475</v>
-      </c>
-      <c r="AF73" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+      <c r="AD73" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE73" t="n">
+        <v>0.0528</v>
+      </c>
+      <c r="AF73" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="AH73" t="n">
@@ -8126,7 +8126,7 @@
         <v>3</v>
       </c>
       <c r="AJ73" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="AK73" t="inlineStr">
         <is>
@@ -8324,7 +8324,7 @@
         <v>5</v>
       </c>
       <c r="Z75" t="n">
-        <v>0.519</v>
+        <v>1</v>
       </c>
       <c r="AA75" t="inlineStr">
         <is>
@@ -8352,7 +8352,7 @@
         <v>6</v>
       </c>
       <c r="AJ75" t="n">
-        <v>0.594</v>
+        <v>0.792</v>
       </c>
       <c r="AK75" t="inlineStr">
         <is>
@@ -8550,7 +8550,7 @@
         <v>7</v>
       </c>
       <c r="Z77" t="n">
-        <v>0.414</v>
+        <v>0.368</v>
       </c>
       <c r="AA77" t="inlineStr">
         <is>
@@ -8564,7 +8564,7 @@
         <v>5</v>
       </c>
       <c r="AE77" t="n">
-        <v>0.153</v>
+        <v>0.163</v>
       </c>
       <c r="AF77" t="inlineStr">
         <is>
@@ -8578,7 +8578,7 @@
         <v>2</v>
       </c>
       <c r="AJ77" t="n">
-        <v>0.17</v>
+        <v>0.136</v>
       </c>
       <c r="AK77" t="inlineStr">
         <is>
@@ -8663,7 +8663,7 @@
         <v>9</v>
       </c>
       <c r="Z78" t="n">
-        <v>0.84</v>
+        <v>0.747</v>
       </c>
       <c r="AA78" t="inlineStr">
         <is>
@@ -8677,7 +8677,7 @@
         <v>8</v>
       </c>
       <c r="AE78" t="n">
-        <v>0.582</v>
+        <v>0.544</v>
       </c>
       <c r="AF78" t="inlineStr">
         <is>
@@ -8691,7 +8691,7 @@
         <v>10</v>
       </c>
       <c r="AJ78" t="n">
-        <v>0.325</v>
+        <v>0.304</v>
       </c>
       <c r="AK78" t="inlineStr">
         <is>
@@ -8917,7 +8917,7 @@
         <v>13</v>
       </c>
       <c r="AJ80" t="n">
-        <v>0.423</v>
+        <v>0.451</v>
       </c>
       <c r="AK80" t="inlineStr">
         <is>
@@ -9030,7 +9030,7 @@
         <v>4</v>
       </c>
       <c r="AJ81" t="n">
-        <v>0.229</v>
+        <v>0.204</v>
       </c>
       <c r="AK81" t="inlineStr">
         <is>
@@ -9129,7 +9129,7 @@
         <v>10</v>
       </c>
       <c r="AE82" t="n">
-        <v>0.721</v>
+        <v>0.769</v>
       </c>
       <c r="AF82" t="inlineStr">
         <is>
@@ -9143,7 +9143,7 @@
         <v>9</v>
       </c>
       <c r="AJ82" t="n">
-        <v>0.339</v>
+        <v>0.452</v>
       </c>
       <c r="AK82" t="inlineStr">
         <is>
@@ -9242,7 +9242,7 @@
         <v>9</v>
       </c>
       <c r="AE83" t="n">
-        <v>0.548</v>
+        <v>0.582</v>
       </c>
       <c r="AF83" t="inlineStr">
         <is>
@@ -9355,7 +9355,7 @@
         <v>6</v>
       </c>
       <c r="AE84" t="n">
-        <v>0.999</v>
+        <v>1</v>
       </c>
       <c r="AF84" t="inlineStr">
         <is>
@@ -9369,7 +9369,7 @@
         <v>1</v>
       </c>
       <c r="AJ84" t="n">
-        <v>0.301</v>
+        <v>0.402</v>
       </c>
       <c r="AK84" t="inlineStr">
         <is>
@@ -9454,7 +9454,7 @@
         <v>10</v>
       </c>
       <c r="Z85" t="n">
-        <v>0.744</v>
+        <v>0.829</v>
       </c>
       <c r="AA85" t="inlineStr">
         <is>
@@ -9468,7 +9468,7 @@
         <v>3</v>
       </c>
       <c r="AE85" t="n">
-        <v>0.184</v>
+        <v>0.204</v>
       </c>
       <c r="AF85" t="inlineStr">
         <is>
@@ -9482,7 +9482,7 @@
         <v>12</v>
       </c>
       <c r="AJ85" t="n">
-        <v>0.503</v>
+        <v>0.447</v>
       </c>
       <c r="AK85" t="inlineStr">
         <is>
@@ -9567,7 +9567,7 @@
         <v>4</v>
       </c>
       <c r="Z86" t="n">
-        <v>0.156</v>
+        <v>0.13</v>
       </c>
       <c r="AA86" t="inlineStr">
         <is>
@@ -9581,7 +9581,7 @@
         <v>2</v>
       </c>
       <c r="AE86" t="n">
-        <v>0.08260000000000001</v>
+        <v>0.0689</v>
       </c>
       <c r="AF86" t="inlineStr">
         <is>
@@ -9680,7 +9680,7 @@
         <v>1</v>
       </c>
       <c r="Z87" s="4" t="n">
-        <v>0.047</v>
+        <v>0.0392</v>
       </c>
       <c r="AA87" s="4" t="inlineStr">
         <is>
@@ -9694,7 +9694,7 @@
         <v>4</v>
       </c>
       <c r="AE87" t="n">
-        <v>0.202</v>
+        <v>0.168</v>
       </c>
       <c r="AF87" t="inlineStr">
         <is>
@@ -9793,7 +9793,7 @@
         <v>6</v>
       </c>
       <c r="Z89" t="n">
-        <v>0.439</v>
+        <v>0.468</v>
       </c>
       <c r="AA89" t="inlineStr">
         <is>
@@ -9807,7 +9807,7 @@
         <v>1</v>
       </c>
       <c r="AE89" s="3" t="n">
-        <v>0.00249</v>
+        <v>0.00332</v>
       </c>
       <c r="AF89" s="3" t="inlineStr">
         <is>
@@ -9821,7 +9821,7 @@
         <v>1</v>
       </c>
       <c r="AJ89" s="3" t="n">
-        <v>2.73e-06</v>
+        <v>1.82e-06</v>
       </c>
       <c r="AK89" s="3" t="inlineStr">
         <is>
@@ -9906,7 +9906,7 @@
         <v>2</v>
       </c>
       <c r="Z90" s="4" t="n">
-        <v>0.0203</v>
+        <v>0.0226</v>
       </c>
       <c r="AA90" s="4" t="inlineStr">
         <is>
@@ -10033,7 +10033,7 @@
         <v>13</v>
       </c>
       <c r="AE91" t="n">
-        <v>0.93</v>
+        <v>0.992</v>
       </c>
       <c r="AF91" t="inlineStr">
         <is>
@@ -10047,7 +10047,7 @@
         <v>9</v>
       </c>
       <c r="AJ91" t="n">
-        <v>0.792</v>
+        <v>0.704</v>
       </c>
       <c r="AK91" t="inlineStr">
         <is>
@@ -10146,7 +10146,7 @@
         <v>8</v>
       </c>
       <c r="AE92" t="n">
-        <v>0.544</v>
+        <v>0.726</v>
       </c>
       <c r="AF92" t="inlineStr">
         <is>
@@ -10160,7 +10160,7 @@
         <v>11</v>
       </c>
       <c r="AJ92" t="n">
-        <v>0.878</v>
+        <v>0.976</v>
       </c>
       <c r="AK92" t="inlineStr">
         <is>
@@ -10259,7 +10259,7 @@
         <v>6</v>
       </c>
       <c r="AE93" t="n">
-        <v>0.373</v>
+        <v>0.497</v>
       </c>
       <c r="AF93" t="inlineStr">
         <is>
@@ -10273,7 +10273,7 @@
         <v>7</v>
       </c>
       <c r="AJ93" t="n">
-        <v>0.09810000000000001</v>
+        <v>0.0654</v>
       </c>
       <c r="AK93" t="inlineStr">
         <is>
@@ -10358,7 +10358,7 @@
         <v>4</v>
       </c>
       <c r="Z94" t="n">
-        <v>0.138</v>
+        <v>0.092</v>
       </c>
       <c r="AA94" t="inlineStr">
         <is>
@@ -10386,7 +10386,7 @@
         <v>3</v>
       </c>
       <c r="AJ94" s="3" t="n">
-        <v>8.46e-05</v>
+        <v>5.64e-05</v>
       </c>
       <c r="AK94" s="3" t="inlineStr">
         <is>
@@ -10471,7 +10471,7 @@
         <v>8</v>
       </c>
       <c r="Z95" t="n">
-        <v>0.84</v>
+        <v>0.747</v>
       </c>
       <c r="AA95" t="inlineStr">
         <is>
@@ -10499,7 +10499,7 @@
         <v>2</v>
       </c>
       <c r="AJ95" s="3" t="n">
-        <v>1.88e-05</v>
+        <v>1.25e-05</v>
       </c>
       <c r="AK95" s="3" t="inlineStr">
         <is>
@@ -10584,7 +10584,7 @@
         <v>3</v>
       </c>
       <c r="Z96" t="n">
-        <v>0.118</v>
+        <v>0.0786</v>
       </c>
       <c r="AA96" t="inlineStr">
         <is>
@@ -10697,7 +10697,7 @@
         <v>1</v>
       </c>
       <c r="Z97" s="3" t="n">
-        <v>0.00611</v>
+        <v>0.00407</v>
       </c>
       <c r="AA97" s="3" t="inlineStr">
         <is>
@@ -10711,7 +10711,7 @@
         <v>12</v>
       </c>
       <c r="AE97" t="n">
-        <v>0.858</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="AF97" t="inlineStr">
         <is>
@@ -10725,7 +10725,7 @@
         <v>4</v>
       </c>
       <c r="AJ97" s="3" t="n">
-        <v>0.000256</v>
+        <v>0.00017</v>
       </c>
       <c r="AK97" s="3" t="inlineStr">
         <is>
@@ -10923,7 +10923,7 @@
         <v>5</v>
       </c>
       <c r="Z99" t="n">
-        <v>0.236</v>
+        <v>0.315</v>
       </c>
       <c r="AA99" t="inlineStr">
         <is>
@@ -10937,7 +10937,7 @@
         <v>3</v>
       </c>
       <c r="AE99" t="n">
-        <v>0.17</v>
+        <v>0.113</v>
       </c>
       <c r="AF99" t="inlineStr">
         <is>
@@ -11050,7 +11050,7 @@
         <v>5</v>
       </c>
       <c r="AE100" t="n">
-        <v>0.279</v>
+        <v>0.305</v>
       </c>
       <c r="AF100" t="inlineStr">
         <is>
@@ -11064,7 +11064,7 @@
         <v>5</v>
       </c>
       <c r="AJ100" s="3" t="n">
-        <v>0.000356</v>
+        <v>0.000238</v>
       </c>
       <c r="AK100" s="3" t="inlineStr">
         <is>
@@ -11262,7 +11262,7 @@
         <v>11</v>
       </c>
       <c r="Z102" t="n">
-        <v>0.777</v>
+        <v>0.829</v>
       </c>
       <c r="AA102" t="inlineStr">
         <is>
@@ -11290,7 +11290,7 @@
         <v>6</v>
       </c>
       <c r="AJ102" s="3" t="n">
-        <v>0.000664</v>
+        <v>0.000443</v>
       </c>
       <c r="AK102" s="3" t="inlineStr">
         <is>
@@ -11403,7 +11403,7 @@
         <v>8</v>
       </c>
       <c r="AJ103" t="n">
-        <v>0.408</v>
+        <v>0.363</v>
       </c>
       <c r="AK103" t="inlineStr">
         <is>
@@ -11488,7 +11488,7 @@
         <v>9</v>
       </c>
       <c r="Z104" t="n">
-        <v>0.725</v>
+        <v>0.773</v>
       </c>
       <c r="AA104" t="inlineStr">
         <is>
@@ -11502,7 +11502,7 @@
         <v>14</v>
       </c>
       <c r="AE104" t="n">
-        <v>0.962</v>
+        <v>1</v>
       </c>
       <c r="AF104" t="inlineStr">
         <is>

</xml_diff>